<commit_message>
After XAI setting and creating a web page. Final touches
</commit_message>
<xml_diff>
--- a/classrooms_import.xlsx
+++ b/classrooms_import.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yusuf Yazici\Desktop\OptiClass--An-Integrated-University-Scheduling-and-XAI-Driven-Calendar-Portal-Berkay\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{930F5C39-4FC6-4A4F-B084-5EFD55E6566F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CEBFDB6-7D33-43EE-AFF1-8DC1C3777CE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -469,7 +469,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>30</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -477,7 +477,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>35</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -485,7 +485,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>25</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -493,7 +493,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>20</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -501,7 +501,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>30</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -509,7 +509,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>35</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
@@ -517,7 +517,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>30</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
@@ -525,7 +525,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>25</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
@@ -533,7 +533,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>28</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
@@ -541,7 +541,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>20</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -549,7 +549,7 @@
         <v>12</v>
       </c>
       <c r="B12">
-        <v>30</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
@@ -557,7 +557,7 @@
         <v>13</v>
       </c>
       <c r="B13">
-        <v>30</v>
+        <v>65</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
@@ -565,7 +565,7 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <v>35</v>
+        <v>60</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
@@ -573,7 +573,7 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <v>25</v>
+        <v>65</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
@@ -581,7 +581,7 @@
         <v>16</v>
       </c>
       <c r="B16">
-        <v>20</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
@@ -589,7 +589,7 @@
         <v>17</v>
       </c>
       <c r="B17">
-        <v>30</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
@@ -597,7 +597,7 @@
         <v>18</v>
       </c>
       <c r="B18">
-        <v>35</v>
+        <v>65</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
@@ -605,7 +605,7 @@
         <v>19</v>
       </c>
       <c r="B19">
-        <v>30</v>
+        <v>60</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
@@ -613,7 +613,7 @@
         <v>20</v>
       </c>
       <c r="B20">
-        <v>25</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
@@ -621,7 +621,7 @@
         <v>21</v>
       </c>
       <c r="B21">
-        <v>28</v>
+        <v>50</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
@@ -629,7 +629,7 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>20</v>
+        <v>60</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
@@ -637,7 +637,7 @@
         <v>23</v>
       </c>
       <c r="B23">
-        <v>30</v>
+        <v>60</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
@@ -645,7 +645,7 @@
         <v>24</v>
       </c>
       <c r="B24">
-        <v>30</v>
+        <v>50</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
@@ -653,7 +653,7 @@
         <v>25</v>
       </c>
       <c r="B25">
-        <v>35</v>
+        <v>55</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
@@ -661,7 +661,7 @@
         <v>26</v>
       </c>
       <c r="B26">
-        <v>25</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
@@ -669,7 +669,7 @@
         <v>27</v>
       </c>
       <c r="B27">
-        <v>20</v>
+        <v>45</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
@@ -677,7 +677,7 @@
         <v>28</v>
       </c>
       <c r="B28">
-        <v>30</v>
+        <v>45</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
@@ -685,7 +685,7 @@
         <v>29</v>
       </c>
       <c r="B29">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
21.05.2026 Change happened for web side showing blocked slots in calendar schedule
</commit_message>
<xml_diff>
--- a/classrooms_import.xlsx
+++ b/classrooms_import.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yusuf Yazici\Desktop\OptiClass--An-Integrated-University-Scheduling-and-XAI-Driven-Calendar-Portal-Berkay\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CEBFDB6-7D33-43EE-AFF1-8DC1C3777CE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FE8AB56-6CA3-47D4-B18D-E2624BD8CFA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>Classroom Code</t>
   </si>
@@ -110,6 +110,9 @@
   </si>
   <si>
     <t>Metaverse Lab</t>
+  </si>
+  <si>
+    <t>Z09</t>
   </si>
 </sst>
 </file>
@@ -449,7 +452,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -509,7 +512,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>45</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
@@ -517,7 +520,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>70</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
@@ -525,7 +528,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>70</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
@@ -533,7 +536,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
@@ -541,7 +544,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>60</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -549,7 +552,7 @@
         <v>12</v>
       </c>
       <c r="B12">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
@@ -557,7 +560,7 @@
         <v>13</v>
       </c>
       <c r="B13">
-        <v>65</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
@@ -565,7 +568,7 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <v>60</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
@@ -573,7 +576,7 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <v>65</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
@@ -581,7 +584,7 @@
         <v>16</v>
       </c>
       <c r="B16">
-        <v>70</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
@@ -589,7 +592,7 @@
         <v>17</v>
       </c>
       <c r="B17">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
@@ -597,7 +600,7 @@
         <v>18</v>
       </c>
       <c r="B18">
-        <v>65</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
@@ -605,7 +608,7 @@
         <v>19</v>
       </c>
       <c r="B19">
-        <v>60</v>
+        <v>90</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
@@ -613,7 +616,7 @@
         <v>20</v>
       </c>
       <c r="B20">
-        <v>55</v>
+        <v>45</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
@@ -621,7 +624,7 @@
         <v>21</v>
       </c>
       <c r="B21">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
@@ -629,7 +632,7 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>60</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
@@ -637,7 +640,7 @@
         <v>23</v>
       </c>
       <c r="B23">
-        <v>60</v>
+        <v>45</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
@@ -645,7 +648,7 @@
         <v>24</v>
       </c>
       <c r="B24">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
@@ -653,7 +656,7 @@
         <v>25</v>
       </c>
       <c r="B25">
-        <v>55</v>
+        <v>45</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
@@ -661,7 +664,7 @@
         <v>26</v>
       </c>
       <c r="B26">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
@@ -685,7 +688,15 @@
         <v>29</v>
       </c>
       <c r="B29">
-        <v>25</v>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>30</v>
+      </c>
+      <c r="B30">
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>